<commit_message>
Add border support to styles
</commit_message>
<xml_diff>
--- a/test/snap/styles.snap.xlsx
+++ b/test/snap/styles.snap.xlsx
@@ -36,16 +36,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border/>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <top style="double"/>
+    </border>
   </borders>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf fontId="0" applyFont="1"/>
     <xf numFmtId="164" applyNumberFormat="1"/>
     <xf numFmtId="165" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" applyFont="1"/>
     <xf fontId="2"/>
     <xf fontId="0"/>
+    <xf fontId="0" borderId="1" applyBorder="1"/>
+    <xf fontId="0" borderId="2" applyBorder="1"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -85,7 +96,7 @@
           <t>Sized Row</t>
         </is>
       </c>
-      <c r="B3">
+      <c r="B3" s="6">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add fill support to styles
</commit_message>
<xml_diff>
--- a/test/snap/styles.snap.xlsx
+++ b/test/snap/styles.snap.xlsx
@@ -28,12 +28,22 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <bgColor rgb="FF9900"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -48,7 +58,7 @@
       <top style="double"/>
     </border>
   </borders>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf fontId="0" applyFont="1"/>
     <xf numFmtId="164" applyNumberFormat="1"/>
     <xf numFmtId="165" applyNumberFormat="1"/>
@@ -57,13 +67,15 @@
     <xf fontId="0"/>
     <xf fontId="0" borderId="1" applyBorder="1"/>
     <xf fontId="0" borderId="2" applyBorder="1"/>
+    <xf fontId="0" fillId="2" applyFill="1"/>
+    <xf fontId="0" fillId="3" applyFill="1"/>
   </cellXfs>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <cols>
     <col min="1" max="1"/>
   </cols>
@@ -100,6 +112,16 @@
         <v>1</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Filled</t>
+        </is>
+      </c>
+      <c r="B4" s="9">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>